<commit_message>
chg: Updated friendly situation, VID intsum, JFC D&G, weather, ordnance for D6.1
</commit_message>
<xml_diff>
--- a/MISSION INFORMATION/OPAC Ordnance.xlsx
+++ b/MISSION INFORMATION/OPAC Ordnance.xlsx
@@ -856,7 +856,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1041,7 +1041,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1461,7 +1461,7 @@
       <c r="R1" s="80"/>
       <c r="S1" s="80"/>
       <c r="T1" s="72" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="39.75" customHeight="1">
@@ -1798,7 +1798,9 @@
       <c r="J11" s="56"/>
       <c r="K11" s="56"/>
       <c r="L11" s="56"/>
-      <c r="M11" s="56"/>
+      <c r="M11" s="56">
+        <v>2</v>
+      </c>
       <c r="N11" s="56"/>
       <c r="O11" s="56"/>
       <c r="P11" s="56"/>
@@ -1807,7 +1809,7 @@
       <c r="S11" s="57"/>
       <c r="T11" s="71">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1843,7 +1845,9 @@
       <c r="L12" s="59">
         <v>1</v>
       </c>
-      <c r="M12" s="51"/>
+      <c r="M12" s="51">
+        <v>4</v>
+      </c>
       <c r="N12" s="51"/>
       <c r="O12" s="51"/>
       <c r="P12" s="51"/>
@@ -1852,7 +1856,7 @@
       <c r="S12" s="52"/>
       <c r="T12" s="71">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1878,7 +1882,9 @@
       <c r="J13" s="56"/>
       <c r="K13" s="56"/>
       <c r="L13" s="60"/>
-      <c r="M13" s="56"/>
+      <c r="M13" s="56">
+        <v>1</v>
+      </c>
       <c r="N13" s="56"/>
       <c r="O13" s="56"/>
       <c r="P13" s="56"/>
@@ -1887,7 +1893,7 @@
       <c r="S13" s="57"/>
       <c r="T13" s="71">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1950,7 +1956,9 @@
       <c r="L15" s="56">
         <v>6</v>
       </c>
-      <c r="M15" s="56"/>
+      <c r="M15" s="56">
+        <v>7</v>
+      </c>
       <c r="N15" s="56"/>
       <c r="O15" s="56"/>
       <c r="P15" s="56"/>
@@ -1959,7 +1967,7 @@
       <c r="S15" s="57"/>
       <c r="T15" s="71">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -2057,7 +2065,9 @@
       <c r="L18" s="51">
         <v>4</v>
       </c>
-      <c r="M18" s="51"/>
+      <c r="M18" s="51">
+        <v>4</v>
+      </c>
       <c r="N18" s="51"/>
       <c r="O18" s="51"/>
       <c r="P18" s="51"/>
@@ -2066,7 +2076,7 @@
       <c r="S18" s="52"/>
       <c r="T18" s="53">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="15.75" thickBot="1">

</xml_diff>

<commit_message>
chg: Prep for D7 (JFC D&G, Friendly situation .cf, VID INTSUM, Ordnance and weather
</commit_message>
<xml_diff>
--- a/MISSION INFORMATION/OPAC Ordnance.xlsx
+++ b/MISSION INFORMATION/OPAC Ordnance.xlsx
@@ -856,7 +856,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1041,7 +1041,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1461,7 +1461,7 @@
       <c r="R1" s="80"/>
       <c r="S1" s="80"/>
       <c r="T1" s="72" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="39.75" customHeight="1">
@@ -1848,15 +1848,19 @@
       <c r="M12" s="51">
         <v>4</v>
       </c>
-      <c r="N12" s="51"/>
-      <c r="O12" s="51"/>
+      <c r="N12" s="51">
+        <v>3</v>
+      </c>
+      <c r="O12" s="51">
+        <v>2</v>
+      </c>
       <c r="P12" s="51"/>
       <c r="Q12" s="52"/>
       <c r="R12" s="52"/>
       <c r="S12" s="52"/>
       <c r="T12" s="71">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1959,7 +1963,9 @@
       <c r="M15" s="56">
         <v>7</v>
       </c>
-      <c r="N15" s="56"/>
+      <c r="N15" s="56">
+        <v>4</v>
+      </c>
       <c r="O15" s="56"/>
       <c r="P15" s="56"/>
       <c r="Q15" s="57"/>
@@ -1967,7 +1973,7 @@
       <c r="S15" s="57"/>
       <c r="T15" s="71">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -2069,14 +2075,16 @@
         <v>4</v>
       </c>
       <c r="N18" s="51"/>
-      <c r="O18" s="51"/>
+      <c r="O18" s="51">
+        <v>2</v>
+      </c>
       <c r="P18" s="51"/>
       <c r="Q18" s="52"/>
       <c r="R18" s="52"/>
       <c r="S18" s="52"/>
       <c r="T18" s="53">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="15.75" thickBot="1">

</xml_diff>